<commit_message>
Edited Unitmaster and added the component range to the JSON to simplify the data gathring while validation
</commit_message>
<xml_diff>
--- a/refrenceMaterial/unitMaster.xlsx
+++ b/refrenceMaterial/unitMaster.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\khode\Desktop\MPUTESTER\refrenceMaterial\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6266EF55-342A-429A-B969-FB2C288983B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="37">
   <si>
     <t xml:space="preserve">PartNo </t>
   </si>
@@ -61,69 +70,82 @@
     <t>LowerResistance</t>
   </si>
   <si>
-    <t>UpperVoltage</t>
-  </si>
-  <si>
-    <t>LowerVoltage</t>
-  </si>
-  <si>
     <t>UpperInductance</t>
   </si>
   <si>
+    <t>MPU1</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>POWERMATE</t>
+  </si>
+  <si>
+    <t>MPU2</t>
+  </si>
+  <si>
+    <t>MPU3</t>
+  </si>
+  <si>
+    <t>MPU4</t>
+  </si>
+  <si>
+    <t>MPU5</t>
+  </si>
+  <si>
+    <t>MPU6</t>
+  </si>
+  <si>
+    <t>MPU7</t>
+  </si>
+  <si>
+    <t>MPU8</t>
+  </si>
+  <si>
+    <t>MPU9</t>
+  </si>
+  <si>
+    <t>UpperVoltage0kLoad</t>
+  </si>
+  <si>
+    <t>LowerVoltage0kLoad</t>
+  </si>
+  <si>
+    <t>UpperVoltage10kLoad</t>
+  </si>
+  <si>
+    <t>LowerVoltage10kLoad</t>
+  </si>
+  <si>
+    <t>UpperVoltage3k3Load</t>
+  </si>
+  <si>
+    <t>LowerVoltage3k3Load</t>
+  </si>
+  <si>
     <t>LowerInductance</t>
   </si>
   <si>
     <t>FREQUENCY</t>
-  </si>
-  <si>
-    <t>MPU1</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>Normal</t>
-  </si>
-  <si>
-    <t>POWERMATE</t>
-  </si>
-  <si>
-    <t>MPU2</t>
-  </si>
-  <si>
-    <t>MPU3</t>
-  </si>
-  <si>
-    <t>MPU4</t>
-  </si>
-  <si>
-    <t>MPU5</t>
-  </si>
-  <si>
-    <t>MPU6</t>
-  </si>
-  <si>
-    <t>MPU7</t>
-  </si>
-  <si>
-    <t>MPU8</t>
-  </si>
-  <si>
-    <t>MPU9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -134,36 +156,43 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -353,24 +382,28 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Y10"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="6" max="6" width="16.38"/>
-    <col customWidth="1" min="15" max="15" width="13.88"/>
-    <col customWidth="1" min="16" max="16" width="14.63"/>
-    <col customWidth="1" min="19" max="19" width="13.63"/>
-    <col customWidth="1" min="20" max="20" width="14.38"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="15" max="15" width="13.85546875" customWidth="1"/>
+    <col min="16" max="16" width="14.5703125" customWidth="1"/>
+    <col min="19" max="19" width="13.5703125" customWidth="1"/>
+    <col min="20" max="20" width="14.42578125" customWidth="1"/>
+    <col min="24" max="25" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -420,42 +453,54 @@
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="X1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>12345</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1">
-        <v>12345.0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="C2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E2" s="1">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G2" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="H2" s="1">
         <v>0.2</v>
@@ -467,60 +512,72 @@
         <v>0.5</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="L2" s="1">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="O2" s="1">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="P2" s="1">
-        <v>1500.0</v>
+        <v>1500</v>
       </c>
       <c r="Q2" s="1">
-        <v>3456.0</v>
+        <v>3456</v>
       </c>
       <c r="R2" s="1">
-        <v>123.0</v>
+        <v>123</v>
       </c>
       <c r="S2" s="1">
-        <v>2345.0</v>
+        <v>123</v>
       </c>
       <c r="T2" s="1">
-        <v>5678.0</v>
+        <v>123</v>
       </c>
       <c r="U2" s="1">
-        <v>1234.0</v>
+        <v>123</v>
+      </c>
+      <c r="V2" s="1">
+        <v>123</v>
+      </c>
+      <c r="W2" s="1">
+        <v>2345</v>
+      </c>
+      <c r="X2" s="1">
+        <v>5678</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>1234</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
-        <v>12346.0</v>
+        <v>12346</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C3" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E3" s="1">
-        <v>52.0</v>
+        <v>52</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G3" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="H3" s="1">
         <v>0.3</v>
@@ -532,60 +589,72 @@
         <v>0.6</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="L3" s="1">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="O3" s="1">
-        <v>2001.0</v>
+        <v>2001</v>
       </c>
       <c r="P3" s="1">
-        <v>1501.0</v>
+        <v>1501</v>
       </c>
       <c r="Q3" s="1">
-        <v>3457.0</v>
+        <v>3457</v>
       </c>
       <c r="R3" s="1">
-        <v>124.0</v>
+        <v>124</v>
       </c>
       <c r="S3" s="1">
-        <v>2346.0</v>
+        <v>123</v>
       </c>
       <c r="T3" s="1">
-        <v>5679.0</v>
+        <v>123</v>
       </c>
       <c r="U3" s="1">
-        <v>1235.0</v>
+        <v>123</v>
+      </c>
+      <c r="V3" s="1">
+        <v>123</v>
+      </c>
+      <c r="W3" s="1">
+        <v>2346</v>
+      </c>
+      <c r="X3" s="1">
+        <v>5679</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>1234</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
-        <v>12347.0</v>
+        <v>12347</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E4" s="1">
-        <v>54.0</v>
+        <v>54</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G4" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="H4" s="1">
         <v>0.4</v>
@@ -597,60 +666,72 @@
         <v>0.7</v>
       </c>
       <c r="K4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L4" s="1">
+        <v>22</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O4" s="1">
+        <v>2002</v>
+      </c>
+      <c r="P4" s="1">
+        <v>1502</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>3458</v>
+      </c>
+      <c r="R4" s="1">
+        <v>125</v>
+      </c>
+      <c r="S4" s="1">
+        <v>123</v>
+      </c>
+      <c r="T4" s="1">
+        <v>123</v>
+      </c>
+      <c r="U4" s="1">
+        <v>123</v>
+      </c>
+      <c r="V4" s="1">
+        <v>123</v>
+      </c>
+      <c r="W4" s="1">
+        <v>2347</v>
+      </c>
+      <c r="X4" s="1">
+        <v>5680</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>12348</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L4" s="1">
-        <v>22.0</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O4" s="1">
-        <v>2002.0</v>
-      </c>
-      <c r="P4" s="1">
-        <v>1502.0</v>
-      </c>
-      <c r="Q4" s="1">
-        <v>3458.0</v>
-      </c>
-      <c r="R4" s="1">
-        <v>125.0</v>
-      </c>
-      <c r="S4" s="1">
-        <v>2347.0</v>
-      </c>
-      <c r="T4" s="1">
-        <v>5680.0</v>
-      </c>
-      <c r="U4" s="1">
-        <v>1236.0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1">
-        <v>12348.0</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="C5" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E5" s="1">
-        <v>56.0</v>
+        <v>56</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G5" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="H5" s="1">
         <v>0.5</v>
@@ -662,60 +743,72 @@
         <v>0.8</v>
       </c>
       <c r="K5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L5" s="1">
         <v>23</v>
       </c>
-      <c r="L5" s="1">
-        <v>23.0</v>
-      </c>
       <c r="M5" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="N5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O5" s="1">
+        <v>2003</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1503</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>3459</v>
+      </c>
+      <c r="R5" s="1">
+        <v>126</v>
+      </c>
+      <c r="S5" s="1">
+        <v>123</v>
+      </c>
+      <c r="T5" s="1">
+        <v>123</v>
+      </c>
+      <c r="U5" s="1">
+        <v>123</v>
+      </c>
+      <c r="V5" s="1">
+        <v>123</v>
+      </c>
+      <c r="W5" s="1">
+        <v>2348</v>
+      </c>
+      <c r="X5" s="1">
+        <v>5681</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>12349</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O5" s="1">
-        <v>2003.0</v>
-      </c>
-      <c r="P5" s="1">
-        <v>1503.0</v>
-      </c>
-      <c r="Q5" s="1">
-        <v>3459.0</v>
-      </c>
-      <c r="R5" s="1">
-        <v>126.0</v>
-      </c>
-      <c r="S5" s="1">
-        <v>2348.0</v>
-      </c>
-      <c r="T5" s="1">
-        <v>5681.0</v>
-      </c>
-      <c r="U5" s="1">
-        <v>1237.0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1">
-        <v>12349.0</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="C6" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E6" s="1">
-        <v>58.0</v>
+        <v>58</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G6" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="H6" s="1">
         <v>0.6</v>
@@ -727,60 +820,72 @@
         <v>0.9</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="L6" s="1">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="O6" s="1">
-        <v>2004.0</v>
+        <v>2004</v>
       </c>
       <c r="P6" s="1">
-        <v>1504.0</v>
+        <v>1504</v>
       </c>
       <c r="Q6" s="1">
-        <v>3460.0</v>
+        <v>3460</v>
       </c>
       <c r="R6" s="1">
-        <v>127.0</v>
+        <v>127</v>
       </c>
       <c r="S6" s="1">
-        <v>2349.0</v>
+        <v>123</v>
       </c>
       <c r="T6" s="1">
-        <v>5682.0</v>
+        <v>123</v>
       </c>
       <c r="U6" s="1">
-        <v>1238.0</v>
+        <v>123</v>
+      </c>
+      <c r="V6" s="1">
+        <v>123</v>
+      </c>
+      <c r="W6" s="1">
+        <v>2349</v>
+      </c>
+      <c r="X6" s="1">
+        <v>5682</v>
+      </c>
+      <c r="Y6" s="1">
+        <v>1234</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
-        <v>12350.0</v>
+        <v>12350</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C7" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1">
-        <v>60.0</v>
+        <v>60</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G7" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="H7" s="1">
         <v>0.7</v>
@@ -789,63 +894,75 @@
         <v>0.8</v>
       </c>
       <c r="J7" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="L7" s="1">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="O7" s="1">
-        <v>2005.0</v>
+        <v>2005</v>
       </c>
       <c r="P7" s="1">
-        <v>1505.0</v>
+        <v>1505</v>
       </c>
       <c r="Q7" s="1">
-        <v>3461.0</v>
+        <v>3461</v>
       </c>
       <c r="R7" s="1">
-        <v>128.0</v>
+        <v>128</v>
       </c>
       <c r="S7" s="1">
-        <v>2350.0</v>
+        <v>123</v>
       </c>
       <c r="T7" s="1">
-        <v>5683.0</v>
+        <v>123</v>
       </c>
       <c r="U7" s="1">
-        <v>1239.0</v>
+        <v>123</v>
+      </c>
+      <c r="V7" s="1">
+        <v>123</v>
+      </c>
+      <c r="W7" s="1">
+        <v>2350</v>
+      </c>
+      <c r="X7" s="1">
+        <v>5683</v>
+      </c>
+      <c r="Y7" s="1">
+        <v>1234</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
-        <v>12351.0</v>
+        <v>12351</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C8" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E8" s="1">
-        <v>62.0</v>
+        <v>62</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G8" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="H8" s="1">
         <v>0.8</v>
@@ -854,63 +971,75 @@
         <v>0.81</v>
       </c>
       <c r="J8" s="1">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="L8" s="1">
-        <v>26.0</v>
+        <v>26</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="O8" s="1">
-        <v>2006.0</v>
+        <v>2006</v>
       </c>
       <c r="P8" s="1">
-        <v>1506.0</v>
+        <v>1506</v>
       </c>
       <c r="Q8" s="1">
-        <v>3462.0</v>
+        <v>3462</v>
       </c>
       <c r="R8" s="1">
-        <v>129.0</v>
+        <v>129</v>
       </c>
       <c r="S8" s="1">
-        <v>2351.0</v>
+        <v>123</v>
       </c>
       <c r="T8" s="1">
-        <v>5684.0</v>
+        <v>123</v>
       </c>
       <c r="U8" s="1">
-        <v>1240.0</v>
+        <v>123</v>
+      </c>
+      <c r="V8" s="1">
+        <v>123</v>
+      </c>
+      <c r="W8" s="1">
+        <v>2351</v>
+      </c>
+      <c r="X8" s="1">
+        <v>5684</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>1234</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
-        <v>12352.0</v>
+        <v>12352</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C9" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E9" s="1">
-        <v>64.0</v>
+        <v>64</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G9" s="1">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="H9" s="1">
         <v>0.9</v>
@@ -922,63 +1051,75 @@
         <v>1.2</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="L9" s="1">
-        <v>27.0</v>
+        <v>27</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="O9" s="1">
-        <v>2007.0</v>
+        <v>2007</v>
       </c>
       <c r="P9" s="1">
-        <v>1507.0</v>
+        <v>1507</v>
       </c>
       <c r="Q9" s="1">
-        <v>3463.0</v>
+        <v>3463</v>
       </c>
       <c r="R9" s="1">
-        <v>130.0</v>
+        <v>130</v>
       </c>
       <c r="S9" s="1">
-        <v>2352.0</v>
+        <v>123</v>
       </c>
       <c r="T9" s="1">
-        <v>5685.0</v>
+        <v>123</v>
       </c>
       <c r="U9" s="1">
-        <v>1241.0</v>
+        <v>123</v>
+      </c>
+      <c r="V9" s="1">
+        <v>123</v>
+      </c>
+      <c r="W9" s="1">
+        <v>2352</v>
+      </c>
+      <c r="X9" s="1">
+        <v>5685</v>
+      </c>
+      <c r="Y9" s="1">
+        <v>1234</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>12353.0</v>
+        <v>12353</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C10" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E10" s="1">
-        <v>66.0</v>
+        <v>66</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G10" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="H10" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="1">
         <v>0.83</v>
@@ -987,40 +1128,52 @@
         <v>1.3</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="L10" s="1">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="O10" s="1">
-        <v>2008.0</v>
+        <v>2008</v>
       </c>
       <c r="P10" s="1">
-        <v>1508.0</v>
+        <v>1508</v>
       </c>
       <c r="Q10" s="1">
-        <v>3464.0</v>
+        <v>3464</v>
       </c>
       <c r="R10" s="1">
-        <v>131.0</v>
+        <v>131</v>
       </c>
       <c r="S10" s="1">
-        <v>2353.0</v>
+        <v>123</v>
       </c>
       <c r="T10" s="1">
-        <v>5686.0</v>
+        <v>123</v>
       </c>
       <c r="U10" s="1">
-        <v>1242.0</v>
+        <v>123</v>
+      </c>
+      <c r="V10" s="1">
+        <v>123</v>
+      </c>
+      <c r="W10" s="1">
+        <v>2353</v>
+      </c>
+      <c r="X10" s="1">
+        <v>5686</v>
+      </c>
+      <c r="Y10" s="1">
+        <v>1234</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>